<commit_message>
Fold Cloud-PASS M14 exam SAY
Co-authored-by: shaseaver25 <shannon@tailoredu.org>
</commit_message>
<xml_diff>
--- a/teaching-pack/18-M14-exam-1-overweight-permit/M14-exam-evidence.xlsx
+++ b/teaching-pack/18-M14-exam-1-overweight-permit/M14-exam-evidence.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REVIEW_BASIS" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'START_HERE'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'START_HERE'!$A$1:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'PERMIT_REQUEST'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CONTROL_GAUGE_TEST'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'REVIEW_BASIS'!$A$1:$C$6</definedName>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -458,113 +458,125 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>exam</t>
+          <t>release_status</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SEIS 201 Exam 1 · M14</t>
+          <t>READY FOR SHANNON SKIM · NOT LMS PUBLISHED</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>job</t>
+          <t>exam</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Otter Bend Lift Bridge · ACMEJOB Unit 2</t>
+          <t>SEIS 201 Exam 1 · M14</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>job</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Internal screening recommendation for one requested night crossing</t>
+          <t>Otter Bend Lift Bridge · ACMEJOB Unit 2</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>time limit</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>75 minutes</t>
+          <t>Internal screening recommendation for one requested night crossing</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>test load</t>
+          <t>time limit</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>80 kip</t>
+          <t>75 minutes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>requested permit load</t>
+          <t>test load</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>104 kip</t>
+          <t>80 kip</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>instructional screening trigger</t>
+          <t>requested permit load</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>240 microstrain</t>
+          <t>104 kip</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>scope</t>
+          <t>instructional screening trigger</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Use only the supplied clean exam file and FOREMAN recommendation.</t>
+          <t>240 microstrain</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Use only the supplied clean exam file and FOREMAN recommendation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>professional boundary</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>This fictional trigger is not a legal permit criterion or bridge capacity rating.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Revert "Fold Cloud-PASS M14 exam SAY"
This reverts commit 5710d69eee49c5d1a82d40e4050057d216c1c2ac.
</commit_message>
<xml_diff>
--- a/teaching-pack/18-M14-exam-1-overweight-permit/M14-exam-evidence.xlsx
+++ b/teaching-pack/18-M14-exam-1-overweight-permit/M14-exam-evidence.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REVIEW_BASIS" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'START_HERE'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'START_HERE'!$A$1:$B$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'PERMIT_REQUEST'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CONTROL_GAUGE_TEST'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'REVIEW_BASIS'!$A$1:$C$6</definedName>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -458,125 +458,113 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>release_status</t>
+          <t>exam</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>READY FOR SHANNON SKIM · NOT LMS PUBLISHED</t>
+          <t>SEIS 201 Exam 1 · M14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>exam</t>
+          <t>job</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>SEIS 201 Exam 1 · M14</t>
+          <t>Otter Bend Lift Bridge · ACMEJOB Unit 2</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>job</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Otter Bend Lift Bridge · ACMEJOB Unit 2</t>
+          <t>Internal screening recommendation for one requested night crossing</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>time limit</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Internal screening recommendation for one requested night crossing</t>
+          <t>75 minutes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>time limit</t>
+          <t>test load</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>75 minutes</t>
+          <t>80 kip</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>test load</t>
+          <t>requested permit load</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>80 kip</t>
+          <t>104 kip</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>requested permit load</t>
+          <t>instructional screening trigger</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>104 kip</t>
+          <t>240 microstrain</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>instructional screening trigger</t>
+          <t>scope</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>240 microstrain</t>
+          <t>Use only the supplied clean exam file and FOREMAN recommendation.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>scope</t>
+          <t>professional boundary</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Use only the supplied clean exam file and FOREMAN recommendation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>professional boundary</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
           <t>This fictional trigger is not a legal permit criterion or bridge capacity rating.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B11"/>
+  <autoFilter ref="A1:B10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Reapply "Fold Cloud-PASS M14 exam SAY"
This reverts commit d2434907d0376321689dd9e707e758c2950ce26c.
</commit_message>
<xml_diff>
--- a/teaching-pack/18-M14-exam-1-overweight-permit/M14-exam-evidence.xlsx
+++ b/teaching-pack/18-M14-exam-1-overweight-permit/M14-exam-evidence.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REVIEW_BASIS" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'START_HERE'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'START_HERE'!$A$1:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'PERMIT_REQUEST'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CONTROL_GAUGE_TEST'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'REVIEW_BASIS'!$A$1:$C$6</definedName>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -458,113 +458,125 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>exam</t>
+          <t>release_status</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SEIS 201 Exam 1 · M14</t>
+          <t>READY FOR SHANNON SKIM · NOT LMS PUBLISHED</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>job</t>
+          <t>exam</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Otter Bend Lift Bridge · ACMEJOB Unit 2</t>
+          <t>SEIS 201 Exam 1 · M14</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>decision</t>
+          <t>job</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Internal screening recommendation for one requested night crossing</t>
+          <t>Otter Bend Lift Bridge · ACMEJOB Unit 2</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>time limit</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>75 minutes</t>
+          <t>Internal screening recommendation for one requested night crossing</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>test load</t>
+          <t>time limit</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>80 kip</t>
+          <t>75 minutes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>requested permit load</t>
+          <t>test load</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>104 kip</t>
+          <t>80 kip</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>instructional screening trigger</t>
+          <t>requested permit load</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>240 microstrain</t>
+          <t>104 kip</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>scope</t>
+          <t>instructional screening trigger</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Use only the supplied clean exam file and FOREMAN recommendation.</t>
+          <t>240 microstrain</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Use only the supplied clean exam file and FOREMAN recommendation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>professional boundary</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>This fictional trigger is not a legal permit criterion or bridge capacity rating.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>